<commit_message>
updated readme, added github publish service
</commit_message>
<xml_diff>
--- a/services/data_raw/eurostat/AT_cars_road_eqr_carpda.xlsx
+++ b/services/data_raw/eurostat/AT_cars_road_eqr_carpda.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,89 +417,89 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>freq</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mot_nrg</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>geo\TIME_PERIOD</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -572,7 +560,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -587,7 +575,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Petroleum products [PET]</t>
+          <t>Petrol [PET]</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -633,7 +621,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -692,7 +680,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -753,7 +741,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -814,7 +802,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -875,7 +863,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -936,7 +924,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -997,7 +985,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -1058,7 +1046,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -1119,7 +1107,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -1180,7 +1168,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1241,7 +1229,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1302,7 +1290,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -1363,7 +1351,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -1412,7 +1400,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -1461,7 +1449,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -1522,7 +1510,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
       <c r="B19" t="inlineStr">

</xml_diff>